<commit_message>
BGSC, BGBSC move start year
</commit_message>
<xml_diff>
--- a/InputData/endo-learn/BCSG/BAU CO2 Sequestered Globally.xlsx
+++ b/InputData/endo-learn/BCSG/BAU CO2 Sequestered Globally.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\endo-learn\BCSG\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OliviaAshmoore\Documents\Github Repos\eps-us\InputData\endo-learn\BCSG\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60A4F206-FF00-4F41-A2CB-11CEB5899944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47CCF514-30E3-459B-A2FF-9A648C4225AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="450" yWindow="210" windowWidth="18480" windowHeight="17100" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -861,22 +861,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="38.7265625" customWidth="1"/>
+    <col min="2" max="2" width="38.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -884,62 +884,62 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B5" s="12">
         <v>2017</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B7" s="13" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -956,21 +956,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A15:AN27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.1796875" customWidth="1"/>
+    <col min="1" max="1" width="28.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.140625" customWidth="1"/>
     <col min="3" max="8" width="12" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="13.1796875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="10" max="13" width="13.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="15" spans="1:1" ht="23.5" x14ac:dyDescent="0.55000000000000004">
+    <row r="15" spans="1:1" ht="23.25" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="1:40" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:40" ht="18" x14ac:dyDescent="0.35">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="18" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>4</v>
       </c>
@@ -1232,7 +1232,7 @@
         <v>645.25886199836145</v>
       </c>
     </row>
-    <row r="19" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>5</v>
       </c>
@@ -1378,7 +1378,7 @@
         <v>140.98274447844116</v>
       </c>
     </row>
-    <row r="20" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>6</v>
       </c>
@@ -1524,7 +1524,7 @@
         <v>133.61743935810051</v>
       </c>
     </row>
-    <row r="21" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A21" s="9" t="s">
         <v>7</v>
       </c>
@@ -1670,7 +1670,7 @@
         <v>919.8590458349031</v>
       </c>
     </row>
-    <row r="23" spans="1:40" ht="16.5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:40" ht="18" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>8</v>
       </c>
@@ -1786,7 +1786,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="24" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>4</v>
       </c>
@@ -1934,7 +1934,7 @@
       <c r="AM24" s="5"/>
       <c r="AN24" s="5"/>
     </row>
-    <row r="25" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>5</v>
       </c>
@@ -2082,7 +2082,7 @@
       <c r="AM25" s="5"/>
       <c r="AN25" s="5"/>
     </row>
-    <row r="26" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>6</v>
       </c>
@@ -2230,7 +2230,7 @@
       <c r="AM26" s="5"/>
       <c r="AN26" s="5"/>
     </row>
-    <row r="27" spans="1:40" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:40" x14ac:dyDescent="0.25">
       <c r="A27" s="9" t="s">
         <v>7</v>
       </c>
@@ -2390,12 +2390,12 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:AB2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="43.453125" customWidth="1"/>
+    <col min="1" max="1" width="43.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:28" x14ac:dyDescent="0.25">
       <c r="B1">
         <v>2024</v>
       </c>
@@ -2478,7 +2478,7 @@
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:28" ht="30" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>21</v>
       </c>
@@ -2602,23 +2602,23 @@
     <tabColor theme="8" tint="-0.249977111117893"/>
   </sheetPr>
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20.1796875" customWidth="1"/>
+    <col min="1" max="1" width="20.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="B1">
-        <v>2023</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="43.5" x14ac:dyDescent="0.35">
+        <v>2024</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="60" x14ac:dyDescent="0.25">
       <c r="A2" s="14" t="s">
         <v>21</v>
       </c>
       <c r="B2" s="11">
-        <f>Data!K21*10^6</f>
-        <v>246996767.7401211</v>
+        <f>BCSG!B2</f>
+        <v>274440853.04457903</v>
       </c>
     </row>
   </sheetData>

</xml_diff>